<commit_message>
Update the public demo: 13 cross-pollination analyses with evidence landscape and learning cards, corrected federal counts and wording, API guide
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/downloads/Q5Ml2-H9W7dHXMRqoUQhlngk.xlsx
+++ b/data/downloads/Q5Ml2-H9W7dHXMRqoUQhlngk.xlsx
@@ -5424,7 +5424,7 @@
       </c>
       <c r="F15" s="1" t="inlineStr">
         <is>
-          <t>Raw algorithm-identified PASC prevalence among COVID-19 cases (2020-2023): the document reports 28.5% as the share of adults who ever had COVID-19 that ever experienced Long COVID; the national survey's 18 wave(s) in that period ranged from 25.6% to 35.1% (interval bounds 24.9% to 36%), so the document's figure is inside the published 95% interval of at least one survey wave. The survey is self-reported adults; a different definition or population in the document makes a gap expected, so treat it as a prompt to check. Federal source: household survey (self-report), 2022-2024; computed in code from the federal file; no AI model.</t>
+          <t>Raw algorithm-identified PASC prevalence among COVID-19 cases (2020-2023): the document reports 28.5% as the share of adults who ever had COVID-19 that ever experienced Long COVID; the national survey's 18 wave(s) in that period ranged from 25.6% to 35.1% (interval bounds 24.9% to 36%), so the document's figure is inside the published 95% interval of at least one survey wave. The survey is self-reported adults; a different definition or population in the document makes a gap expected, so treat it as a prompt to check. The document's figure is for "Massachusetts (MGB health system)", not the whole United States, so the national survey is context only here, not a like-for-like comparison. The survey has no data for 2020, 2021. Federal source: household survey (self-report), 2022-2024; computed in code from the federal file; no AI model.</t>
         </is>
       </c>
     </row>
@@ -5452,7 +5452,7 @@
       </c>
       <c r="F16" s="1" t="inlineStr">
         <is>
-          <t>PPV-adjusted PASC prevalence estimate (2020-2023): the document reports 22.8% as the share of adults who ever had COVID-19 that ever experienced Long COVID; the national survey's 18 wave(s) in that period ranged from 25.6% to 35.1% (interval bounds 24.9% to 36%), so the document's figure is below every survey wave interval in that period. The survey is self-reported adults; a different definition or population in the document makes a gap expected, so treat it as a prompt to check. Federal source: household survey (self-report), 2022-2024; computed in code from the federal file; no AI model.</t>
+          <t>PPV-adjusted PASC prevalence estimate (2020-2023): the document reports 22.8% as the share of adults who ever had COVID-19 that ever experienced Long COVID; the national survey's 18 wave(s) in that period ranged from 25.6% to 35.1% (interval bounds 24.9% to 36%), so the document's figure is below every survey wave interval in that period. The survey is self-reported adults; a different definition or population in the document makes a gap expected, so treat it as a prompt to check. The document's figure is for "Massachusetts (MGB health system)", not the whole United States, so the national survey is context only here, not a like-for-like comparison. The survey has no data for 2020, 2021. Federal source: household survey (self-report), 2022-2024; computed in code from the federal file; no AI model.</t>
         </is>
       </c>
     </row>
@@ -5480,7 +5480,7 @@
       </c>
       <c r="F17" s="1" t="inlineStr">
         <is>
-          <t>NCHS Household Pulse Survey PASC prevalence estimate for Massachusetts (cited by document for comparison) (2022-2023): the document reports 24% as the share of adults who ever had COVID-19 that ever experienced Long COVID; the national survey's 18 wave(s) in that period ranged from 25.6% to 35.1% (interval bounds 24.9% to 36%), so the document's figure is below every survey wave interval in that period. The survey is self-reported adults; a different definition or population in the document makes a gap expected, so treat it as a prompt to check. Federal source: household survey (self-report), 2022-2024; computed in code from the federal file; no AI model.</t>
+          <t>NCHS Household Pulse Survey PASC prevalence estimate for Massachusetts (cited by document for comparison) (2022-2023): the document reports 24% as the share of adults who ever had COVID-19 that ever experienced Long COVID; the national survey's 18 wave(s) in that period ranged from 25.6% to 35.1% (interval bounds 24.9% to 36%), so the document's figure is below every survey wave interval in that period. The survey is self-reported adults; a different definition or population in the document makes a gap expected, so treat it as a prompt to check. The document's figure is for "Massachusetts", not the whole United States, so the national survey is context only here, not a like-for-like comparison. Federal source: household survey (self-report), 2022-2024; computed in code from the federal file; no AI model.</t>
         </is>
       </c>
     </row>

</xml_diff>